<commit_message>
added feature to upload photos to fish recorded and display them. Setting added to store drive id for photo storage.
</commit_message>
<xml_diff>
--- a/sheet/Fishing Example Sheet.xlsx
+++ b/sheet/Fishing Example Sheet.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12312" activeTab="6"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12312"/>
   </bookViews>
   <sheets>
     <sheet name="Dips " sheetId="1" r:id="rId1"/>
@@ -6330,24 +6330,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1">
-          <x14:formula1>
-            <xm:f>Validations!$A$2:$A$200</xm:f>
-          </x14:formula1>
-          <xm:sqref>A2:A959</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1">
-          <x14:formula1>
-            <xm:f>Validations!$B$2:$B$999</xm:f>
-          </x14:formula1>
-          <xm:sqref>C2:C959</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
@@ -11370,24 +11352,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>Validations!$B$2:$B$132</xm:f>
-          </x14:formula1>
-          <xm:sqref>C2:C999</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1">
-          <x14:formula1>
-            <xm:f>Validations!$A$2:$A$200</xm:f>
-          </x14:formula1>
-          <xm:sqref>A2:A999</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
@@ -16310,24 +16274,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>Validations!$B$2:$B$132</xm:f>
-          </x14:formula1>
-          <xm:sqref>C2:C979</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1">
-          <x14:formula1>
-            <xm:f>Validations!$A$2:$A$200</xm:f>
-          </x14:formula1>
-          <xm:sqref>A2:A979</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
@@ -22331,30 +22277,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>Validations!$B$2:$B$132</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2:D979</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1">
-          <x14:formula1>
-            <xm:f>Validations!$A$2:$A$200</xm:f>
-          </x14:formula1>
-          <xm:sqref>A2:A979</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1">
-          <x14:formula1>
-            <xm:f>Validations!$C$2:$C$99999</xm:f>
-          </x14:formula1>
-          <xm:sqref>C2:C999</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
@@ -27357,24 +27279,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>Validations!$B$2:$B$132</xm:f>
-          </x14:formula1>
-          <xm:sqref>C2:C979</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1">
-          <x14:formula1>
-            <xm:f>Validations!$A$2:$A$200</xm:f>
-          </x14:formula1>
-          <xm:sqref>A2:A999</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
@@ -34414,30 +34318,7 @@
       <c r="D1000" s="23"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="E2:E999">
-      <formula1>"Evette,Heini"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>Validations!$E$2:$E$999</xm:f>
-          </x14:formula1>
-          <xm:sqref>C2:D1000</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1">
-          <x14:formula1>
-            <xm:f>Validations!$D$2:$D$999</xm:f>
-          </x14:formula1>
-          <xm:sqref>A2:A1000</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 

</xml_diff>